<commit_message>
creacion de columna Valor y herramienta de busqueda
</commit_message>
<xml_diff>
--- a/lista_eventos_vl550.xlsx
+++ b/lista_eventos_vl550.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bizland365-my.sharepoint.com/personal/simon_vargas_bizland_tech/Documents/TAREAS DIARIAS/7_4_26/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bizland365-my.sharepoint.com/personal/simon_vargas_bizland_tech/Documents/val_log_reader/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="104" documentId="8_{DD8B7EEC-4868-4479-A1B2-219F4CF729D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27295E30-3495-490C-921C-ADD5A5126F36}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3CD72D0F-0109-4709-BAE3-D4DAF02C6335}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3CD72D0F-0109-4709-BAE3-D4DAF02C6335}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="83">
   <si>
     <t>ID</t>
   </si>
@@ -249,18 +249,6 @@
   </si>
   <si>
     <t>Mensaje en log</t>
-  </si>
-  <si>
-    <t>Suma</t>
-  </si>
-  <si>
-    <t>Promedio</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>Recuento</t>
   </si>
   <si>
     <t>Significado</t>
@@ -464,7 +452,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -474,8 +462,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -821,14 +808,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>70</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -1241,11 +1228,11 @@
       <c r="A40" s="7">
         <v>39</v>
       </c>
-      <c r="B40" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="C40" s="10" t="s">
-        <v>86</v>
+      <c r="B40" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
@@ -1253,10 +1240,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="C41" s="10" t="s">
-        <v>86</v>
+        <v>73</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
@@ -1264,10 +1251,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="C42" s="10" t="s">
-        <v>86</v>
+        <v>74</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
@@ -1275,10 +1262,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="C43" s="10" t="s">
-        <v>86</v>
+        <v>75</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
@@ -1286,10 +1273,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="C44" s="10" t="s">
-        <v>86</v>
+        <v>76</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
@@ -1297,10 +1284,10 @@
         <v>44</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="C45" s="10" t="s">
-        <v>86</v>
+        <v>77</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
@@ -1308,10 +1295,10 @@
         <v>45</v>
       </c>
       <c r="B46" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C46" s="9" t="s">
         <v>82</v>
-      </c>
-      <c r="C46" s="10" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
@@ -1319,10 +1306,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="C47" s="10" t="s">
-        <v>86</v>
+        <v>79</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
@@ -1330,10 +1317,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C48" s="10" t="s">
-        <v>86</v>
+        <v>80</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
@@ -1341,10 +1328,10 @@
         <v>48</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C49" s="10" t="s">
-        <v>86</v>
+        <v>81</v>
+      </c>
+      <c r="C49" s="9" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modificacion de excel lista eventos
</commit_message>
<xml_diff>
--- a/lista_eventos_vl550.xlsx
+++ b/lista_eventos_vl550.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bizland365-my.sharepoint.com/personal/simon_vargas_bizland_tech/Documents/Documentos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bizland365-my.sharepoint.com/personal/simon_vargas_bizland_tech/Documents/val_log_reader/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{294A4F71-4DCD-457A-B023-B0EE0B28AABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="8_{294A4F71-4DCD-457A-B023-B0EE0B28AABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA374C87-EE9C-42D1-97D3-8C25643486E6}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-48" windowWidth="23256" windowHeight="12456" xr2:uid="{3CD72D0F-0109-4709-BAE3-D4DAF02C6335}"/>
   </bookViews>
@@ -36,47 +36,20 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="101">
   <si>
     <t>ID</t>
   </si>
   <si>
-    <t xml:space="preserve">Checking EMV library initialization cada una hora lo hace </t>
-  </si>
-  <si>
     <t xml:space="preserve"> sMessage: Autenticacion de datos validada y correcta</t>
   </si>
   <si>
-    <t>Se detectó una tarjeta EMV  --&gt;En VL550</t>
-  </si>
-  <si>
-    <t>Se detectó una tarjeta Mifare --&gt;En VL550</t>
-  </si>
-  <si>
     <t>Couldn't find a controller  --&gt;En VL550</t>
   </si>
   <si>
-    <t>appVersion =    --&gt;En VL550</t>
-  </si>
-  <si>
     <t>The reader did not reply or the reply was not expected  --&gt;En VL550</t>
   </si>
   <si>
-    <t>Tarjeta de inspector --&gt;  En VL550</t>
-  </si>
-  <si>
-    <t>Se informa del estado 17 al validador --&gt;En CGI, indica Chofer logeado</t>
-  </si>
-  <si>
-    <t>Name: SERVICE_ID, Value: --&gt;Log VL550 indica N° Servicio</t>
-  </si>
-  <si>
-    <t>payload de QR: --&gt;Pago con QR en log VL550</t>
-  </si>
-  <si>
-    <t>EMV library is operational --&gt;En VL550</t>
-  </si>
-  <si>
     <t>Checking EMV library initialization</t>
   </si>
   <si>
@@ -92,156 +65,75 @@
     <t>Se detectó una tarjeta EMV</t>
   </si>
   <si>
-    <t>======================  FIN  VALIDACIÓN  ======================</t>
-  </si>
-  <si>
     <t>COMPANY:</t>
   </si>
   <si>
-    <t>nro de empresa--&gt;En VL550</t>
-  </si>
-  <si>
     <t>iAppCalEmv_Debit FAILED</t>
   </si>
   <si>
     <t>iAppCalEmv_Debit OK</t>
   </si>
   <si>
-    <t>iAppCalEmv_Debit   exitoso--&gt;En VL550</t>
-  </si>
-  <si>
-    <t>AppCalEmv_Debit falla --&gt;En VL550</t>
-  </si>
-  <si>
-    <t>4 ultimos numeros de tarjeta EMV --&gt;En VL550</t>
-  </si>
-  <si>
     <t>"serial_number":</t>
   </si>
   <si>
-    <t>nro serial de dispositivo validador --&gt;En VL550</t>
-  </si>
-  <si>
     <t>appName =</t>
   </si>
   <si>
-    <t>nombre de la app</t>
-  </si>
-  <si>
     <t>QR Record serialNumber:</t>
   </si>
   <si>
-    <t>QR identificador  --&gt;VL550</t>
-  </si>
-  <si>
     <t>[QRInputProducer][I]return true</t>
   </si>
   <si>
     <t>[TransactionDAOBPCImpl][T]Transaction Successfully stored!</t>
   </si>
   <si>
-    <t>TRANSACCION EXITOSA después de pagar con EMV</t>
-  </si>
-  <si>
     <t>[IntegrisysEMVReader][D]FARE:</t>
   </si>
   <si>
-    <t>tarifa aplicada: --&gt;En VL550</t>
-  </si>
-  <si>
     <t>[IntegrisysEMVReader][D]sExplanation: TRANSACCION EXITOSA</t>
   </si>
   <si>
-    <t>transaccion con tarjeta EMV exitosa</t>
-  </si>
-  <si>
     <t>Name: CONTADOR_BOLETOS, Value:</t>
   </si>
   <si>
-    <t>valor de contador de boletos --&gt;En VL550</t>
-  </si>
-  <si>
     <t>[ConsoleInterpreter][I]t.counter:</t>
   </si>
   <si>
-    <t xml:space="preserve">valor de contador de boletos  --&gt;En Consola   </t>
-  </si>
-  <si>
     <t>[ApplicationProfile][I]========= HW STATUS =========</t>
   </si>
   <si>
-    <t>indica estados de EMV, QR, Mk Eprom</t>
-  </si>
-  <si>
     <t>driver =</t>
   </si>
   <si>
-    <t>numero de legajo del chofer--&gt;Chofer en  VL550</t>
-  </si>
-  <si>
     <t xml:space="preserve">params line = </t>
   </si>
   <si>
-    <t>inicio de lectura de parametros del colectivo (linea, ruta, descripcion,nro de legajo del conductor)</t>
-  </si>
-  <si>
     <t>merchantName:</t>
   </si>
   <si>
-    <t>nombre de la empresa</t>
-  </si>
-  <si>
     <t>Id: 1523, Name: EVENTS_NUMBER, Value:</t>
   </si>
   <si>
-    <t>evento (cobro de tarifa multipago) nro:</t>
-  </si>
-  <si>
     <t>"versionFW":</t>
   </si>
   <si>
-    <t>version de fw de consola CGI</t>
-  </si>
-  <si>
     <t>[OCConnection][T][BKO --&gt;]</t>
   </si>
   <si>
-    <t>currentStage reporte a back officce--&gt; Etapa en Log de VL</t>
-  </si>
-  <si>
     <t>StateOpeningService()</t>
   </si>
   <si>
-    <t>indica que abre el servicio (conductor inicia jornada)</t>
-  </si>
-  <si>
     <t>Id: 779, Name: SERVICE_ID, Value:</t>
   </si>
   <si>
-    <t>indica N° Servicio abierto--&gt;Log VL550 indica N° Servicio</t>
-  </si>
-  <si>
     <t>SET STATE 26</t>
   </si>
   <si>
-    <t>Estado: 26 . Se cierra servicio--&gt;Este N° 26 es el estado de Cerrado VL550</t>
-  </si>
-  <si>
     <t>SET STATE 23</t>
   </si>
   <si>
-    <t>SERVICE_ID</t>
-  </si>
-  <si>
-    <t>====================== INICIO VALIDACION ======================</t>
-  </si>
-  <si>
-    <t>fin de intento de cobro de pasaje --&gt;En VL550</t>
-  </si>
-  <si>
-    <t>inicio de ntento de cobro de pasaje --&gt;En VL550</t>
-  </si>
-  <si>
     <t>Mensaje en log</t>
   </si>
   <si>
@@ -278,9 +170,6 @@
     <t>Tabla:OL id:10  currVersion:</t>
   </si>
   <si>
-    <t>Identificador de tabla y versión</t>
-  </si>
-  <si>
     <t>[InspectorController][I]Tarjeta de inspector en servicio abierto</t>
   </si>
   <si>
@@ -293,9 +182,6 @@
     <t>[InspectorController][I]Cantidad de registros qr cargados:</t>
   </si>
   <si>
-    <t>Cantidad de registros qr cargado</t>
-  </si>
-  <si>
     <t>tarjeta EMV cargada a Inspector</t>
   </si>
   <si>
@@ -305,25 +191,154 @@
     <t>La consola pidio cerrar servicio</t>
   </si>
   <si>
-    <t>Se cierra servicio</t>
-  </si>
-  <si>
     <t>La consola pidio abrir servicio</t>
   </si>
   <si>
-    <t>Se abre servicio</t>
-  </si>
-  <si>
     <t>Estado del validador:</t>
   </si>
   <si>
-    <t>Estado de validador</t>
-  </si>
-  <si>
     <t>chofer logeado</t>
   </si>
   <si>
-    <t>Estado: 23. Se abre servicio--&gt;Este N° 23 es el estado de Abierto VL550</t>
+    <t>contador de boletos</t>
+  </si>
+  <si>
+    <t>estado EMV, QR</t>
+  </si>
+  <si>
+    <t>lectura de parametros del colectivo</t>
+  </si>
+  <si>
+    <t>nombre empresa</t>
+  </si>
+  <si>
+    <t>legajo del chofer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nro. evento </t>
+  </si>
+  <si>
+    <t>version FW CGI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tarjeta de inspector </t>
+  </si>
+  <si>
+    <t>cantidad de registros QR cargado</t>
+  </si>
+  <si>
+    <t>currentStage reporte a back officce</t>
+  </si>
+  <si>
+    <t>Chofer logeado</t>
+  </si>
+  <si>
+    <t>aperura deservicio</t>
+  </si>
+  <si>
+    <t>nro servicio abierto</t>
+  </si>
+  <si>
+    <t>cierre servicio</t>
+  </si>
+  <si>
+    <t>apertura servicio</t>
+  </si>
+  <si>
+    <t>estado validador</t>
+  </si>
+  <si>
+    <t>Estado: 26 . Se cierra servicio</t>
+  </si>
+  <si>
+    <t>Estado: 23. Se abre servicio</t>
+  </si>
+  <si>
+    <t>Tabla:RL id:9  Version</t>
+  </si>
+  <si>
+    <t>Tabla:AL id:11</t>
+  </si>
+  <si>
+    <t>Tabla:CO id:3  Version</t>
+  </si>
+  <si>
+    <t>Tabla:CD id:15  Version</t>
+  </si>
+  <si>
+    <t>Tabla:LR id:23  Version</t>
+  </si>
+  <si>
+    <t>Tabla:RS id:16  Version</t>
+  </si>
+  <si>
+    <t>Tabla:GP id:1  Version</t>
+  </si>
+  <si>
+    <t>Tabla:SG id:20  Version</t>
+  </si>
+  <si>
+    <t>Tabla:LI id:18  Version</t>
+  </si>
+  <si>
+    <t>Tabla:OL id:10  Version</t>
+  </si>
+  <si>
+    <t>chequeo librería EMV (c/1hr)</t>
+  </si>
+  <si>
+    <t>Se detectó una tarjeta Mifare</t>
+  </si>
+  <si>
+    <t>================= INICIO VALIDACION =================</t>
+  </si>
+  <si>
+    <t>=================  FIN  VALIDACIÓN  =================</t>
+  </si>
+  <si>
+    <t>inicio de validación de pago</t>
+  </si>
+  <si>
+    <t>fin de validación de pago</t>
+  </si>
+  <si>
+    <t>nro de empresa</t>
+  </si>
+  <si>
+    <t>EMV pago  exitoso</t>
+  </si>
+  <si>
+    <t>EMV pago fallido</t>
+  </si>
+  <si>
+    <t>4 ultimos numeros de tarjeta EMV</t>
+  </si>
+  <si>
+    <t>nro serial de  VL550</t>
+  </si>
+  <si>
+    <t>version FW de VL</t>
+  </si>
+  <si>
+    <t>[OCConnection][T][BKO --&gt;] {"command":"config_params",</t>
+  </si>
+  <si>
+    <t>datos de comunicación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">identificación de QR </t>
+  </si>
+  <si>
+    <t>validación de pago con QR</t>
+  </si>
+  <si>
+    <t>TRANSACCION EXITOSA pago con EMV</t>
+  </si>
+  <si>
+    <t>librería EMVoperacional</t>
+  </si>
+  <si>
+    <t>tarifa aplicada</t>
   </si>
 </sst>
 </file>
@@ -491,7 +506,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
@@ -503,6 +518,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -520,10 +541,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -843,185 +860,186 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B1D1B55-AF86-45B6-9E5B-2D3BFD69756D}">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="60.36328125" customWidth="1"/>
     <col min="3" max="3" width="78.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>68</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="7">
         <v>2</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="7">
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="7">
         <v>4</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+      <c r="D5" s="11"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="7">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>65</v>
+      <c r="B6" s="12" t="s">
+        <v>84</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="7">
         <v>6</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>18</v>
+      <c r="B7" s="12" t="s">
+        <v>85</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="7">
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="7">
         <v>8</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="7">
         <v>9</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="7">
         <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="7">
         <v>11</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="7">
         <v>12</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="7">
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>26</v>
+        <v>94</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="7">
         <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="7">
         <v>15</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>11</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
@@ -1030,7 +1048,7 @@
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
@@ -1038,10 +1056,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>34</v>
+        <v>98</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
@@ -1050,7 +1068,7 @@
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="3" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
@@ -1058,10 +1076,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
@@ -1069,10 +1087,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>36</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
@@ -1080,10 +1098,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>38</v>
+        <v>98</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
@@ -1091,10 +1109,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
@@ -1102,10 +1120,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
@@ -1113,10 +1131,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
@@ -1124,10 +1142,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
@@ -1135,10 +1153,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
@@ -1146,10 +1164,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
@@ -1157,10 +1175,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
@@ -1168,10 +1186,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
@@ -1179,10 +1197,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>8</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.35">
@@ -1190,10 +1208,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>87</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.35">
@@ -1201,10 +1219,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>83</v>
+        <v>46</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>86</v>
+        <v>48</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.35">
@@ -1212,10 +1230,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>84</v>
+        <v>47</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1223,10 +1241,10 @@
         <v>34</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.35">
@@ -1234,10 +1252,10 @@
         <v>35</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>94</v>
+        <v>53</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.35">
@@ -1245,10 +1263,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.35">
@@ -1256,10 +1274,10 @@
         <v>37</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.35">
@@ -1267,10 +1285,10 @@
         <v>38</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>88</v>
+        <v>50</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>89</v>
+        <v>67</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.35">
@@ -1278,10 +1296,10 @@
         <v>39</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>90</v>
+        <v>51</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.35">
@@ -1289,10 +1307,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>92</v>
+        <v>52</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
@@ -1300,10 +1318,10 @@
         <v>41</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>61</v>
+        <v>30</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
@@ -1311,131 +1329,120 @@
         <v>42</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="7">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>10</v>
+        <v>34</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="7">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="7">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" s="7">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>72</v>
+        <v>37</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" s="7">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="C48" s="9" t="s">
-        <v>80</v>
+        <v>38</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="7">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="C49" s="9" t="s">
-        <v>80</v>
+        <v>39</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="7">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C50" s="9" t="s">
-        <v>80</v>
+        <v>40</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A51" s="7">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C51" s="9" t="s">
-        <v>80</v>
+        <v>41</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="7">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="C52" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C52" s="8" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" s="7">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B53" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="C53" s="9" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A54" s="7">
-        <v>53</v>
-      </c>
-      <c r="B54" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="C54" s="9" t="s">
-        <v>80</v>
+        <v>43</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
excell y ID 6 corregido
</commit_message>
<xml_diff>
--- a/lista_eventos_vl550.xlsx
+++ b/lista_eventos_vl550.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bizland365-my.sharepoint.com/personal/simon_vargas_bizland_tech/Documents/val_log_reader/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="62" documentId="8_{294A4F71-4DCD-457A-B023-B0EE0B28AABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F25ED196-580A-4CB9-9B51-7CF6D22B010E}"/>
+  <xr:revisionPtr revIDLastSave="96" documentId="8_{294A4F71-4DCD-457A-B023-B0EE0B28AABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8319351-2300-42D3-8BB3-AE82D32D8381}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-48" windowWidth="23256" windowHeight="12456" xr2:uid="{3CD72D0F-0109-4709-BAE3-D4DAF02C6335}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="111">
   <si>
     <t>ID</t>
   </si>
@@ -248,12 +248,6 @@
     <t>estado validador</t>
   </si>
   <si>
-    <t>Estado: 26 . Se cierra servicio</t>
-  </si>
-  <si>
-    <t>Estado: 23. Se abre servicio</t>
-  </si>
-  <si>
     <t>Tabla:RL id:9  Version</t>
   </si>
   <si>
@@ -339,6 +333,42 @@
   </si>
   <si>
     <t>tarifa aplicada</t>
+  </si>
+  <si>
+    <t>SET STATE 20</t>
+  </si>
+  <si>
+    <t>SET STATE  21</t>
+  </si>
+  <si>
+    <t>SET STATE 24</t>
+  </si>
+  <si>
+    <t>SET STATE 28</t>
+  </si>
+  <si>
+    <t>Estado: Actualizacion FW</t>
+  </si>
+  <si>
+    <t>Estado: Abierto al Usuario</t>
+  </si>
+  <si>
+    <t>Estado: Bajo consumo</t>
+  </si>
+  <si>
+    <t>Estado: Cerrado</t>
+  </si>
+  <si>
+    <t>Estado: Se abre servicio</t>
+  </si>
+  <si>
+    <t>Estado: Se cierra servicio</t>
+  </si>
+  <si>
+    <t>SET STATE 3</t>
+  </si>
+  <si>
+    <t>Estado: Presente tarjeta</t>
   </si>
 </sst>
 </file>
@@ -860,7 +890,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B1D1B55-AF86-45B6-9E5B-2D3BFD69756D}">
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="60.36328125" customWidth="1"/>
@@ -886,7 +916,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -908,7 +938,7 @@
         <v>7</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -926,10 +956,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -937,10 +967,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>85</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -951,7 +981,7 @@
         <v>9</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -962,7 +992,7 @@
         <v>11</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
@@ -973,7 +1003,7 @@
         <v>10</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -984,7 +1014,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -995,7 +1025,7 @@
         <v>12</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -1006,7 +1036,7 @@
         <v>13</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
@@ -1014,10 +1044,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
@@ -1028,7 +1058,7 @@
         <v>14</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
@@ -1039,7 +1069,7 @@
         <v>15</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
@@ -1059,7 +1089,7 @@
         <v>16</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
@@ -1079,7 +1109,7 @@
         <v>6</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
@@ -1090,7 +1120,7 @@
         <v>17</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
@@ -1101,7 +1131,7 @@
         <v>18</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
@@ -1314,14 +1344,14 @@
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A42" s="5">
+      <c r="A42" s="7">
         <v>41</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>30</v>
+        <v>109</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>70</v>
+        <v>110</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.35">
@@ -1329,10 +1359,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>31</v>
+        <v>99</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>71</v>
+        <v>106</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.35">
@@ -1340,10 +1370,10 @@
         <v>43</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C44" s="9" t="s">
-        <v>72</v>
+        <v>100</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.35">
@@ -1351,21 +1381,21 @@
         <v>44</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C45" s="9" t="s">
-        <v>73</v>
+        <v>31</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A46" s="5">
+      <c r="A46" s="7">
         <v>45</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C46" s="9" t="s">
-        <v>74</v>
+        <v>101</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.35">
@@ -1373,10 +1403,10 @@
         <v>46</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C47" s="9" t="s">
-        <v>75</v>
+        <v>30</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.35">
@@ -1384,10 +1414,10 @@
         <v>47</v>
       </c>
       <c r="B48" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C48" s="8" t="s">
-        <v>76</v>
+        <v>102</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.35">
@@ -1395,21 +1425,21 @@
         <v>48</v>
       </c>
       <c r="B49" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C49" s="8" t="s">
-        <v>77</v>
+        <v>34</v>
+      </c>
+      <c r="C49" s="9" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A50" s="5">
+      <c r="A50" s="7">
         <v>49</v>
       </c>
       <c r="B50" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C50" s="8" t="s">
-        <v>78</v>
+        <v>35</v>
+      </c>
+      <c r="C50" s="9" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.35">
@@ -1417,10 +1447,10 @@
         <v>50</v>
       </c>
       <c r="B51" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C51" s="8" t="s">
-        <v>79</v>
+        <v>36</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.35">
@@ -1428,10 +1458,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="C52" s="8" t="s">
-        <v>80</v>
+        <v>37</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.35">
@@ -1439,10 +1469,65 @@
         <v>52</v>
       </c>
       <c r="B53" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A54" s="7">
+        <v>53</v>
+      </c>
+      <c r="B54" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A55" s="7">
+        <v>54</v>
+      </c>
+      <c r="B55" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A56" s="7">
+        <v>55</v>
+      </c>
+      <c r="B56" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C56" s="8" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A57" s="7">
+        <v>56</v>
+      </c>
+      <c r="B57" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C57" s="8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A58" s="7">
+        <v>57</v>
+      </c>
+      <c r="B58" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="C53" s="8" t="s">
-        <v>81</v>
+      <c r="C58" s="8" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>